<commit_message>
Add sensor-coverage-gap principle to decision matrix methodology
A monitored equipment parameter (e.g. panel temperature) doesn't
necessarily cover the specific failure mode a physical checklist item
exists to catch (e.g. a blown fuse in one circuit). Documents this as
an explicit rule: SKIP requires the sensor to cover the actual failure
mode, not just "a sensor exists" - otherwise the right call is a
reduced-frequency INSPECT. Also separates the two layers of electrical
checks (certified-electrician legal inspection vs. routine internal
staff rounds) and folds in next steps from the Four Towers site visit
(G1 Hotelo/Trend BACnet-OPC question, Visitt API access).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5iYmbaYQR3KfhiBL7MRAY
</commit_message>
<xml_diff>
--- a/building_ops/output/master_decision_matrix.xlsx
+++ b/building_ops/output/master_decision_matrix.xlsx
@@ -5056,7 +5056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5198,270 +5198,346 @@
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>4. הסבר עמודות מפת ההחלטות</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="29" t="inlineStr">
+          <t>4. עיקרון מרכזי: 'יש חיישן' אינו אומר 'אפשר SKIP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="75" customHeight="1">
+      <c r="A19" s="29" t="inlineStr"/>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>לפני שקובעים החלטת SKIP למשימה, לא מספיק לבדוק "האם יש חיישן על הציוד הזה" — צריך לבדוק ספציפית "האם החיישן הקיים באמת מכסה את סוג הכשל שהבדיקה הפיזית המקורית נועדה לתפוס". לדוגמה: חיישן טמפרטורה וסטטוס מפסקים על לוח חשמל לא בהכרח מזהה נתיך שנשרף במעגל ספציפי, קורוזיה, חיבור רופף או ריח שרוף — אלה כשלים שהבדיקה הפיזית הידנית נועדה לתפוס ושהחיישנים הקיימים אינם מכסים בהכרח.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>מסקנה מעשית</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>כשקיים פער כיסוי כזה, ההחלטה הנכונה היא INSPECT (ביקור פיזי בתדירות מופחתת, ממוקד ספציפית במה שהחיישנים לא רואים) ולא SKIP מלא — עד שמתווסף חיישן ייעודי שסוגר את הפער הספציפי (למשל חיישן זרם/רציפות לכל מעגל בנפרד, לא רק טמפ' כללית של הלוח).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="75" customHeight="1">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>הבחנה חשובה נוספת</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>יש להבדיל בין שתי שכבות שונות של בדיקה שקל לבלבל ביניהן: (1) בדיקה שנתית ע"י גורם מוסמך חיצוני (למשל בודק חשמל מוסמך) — זו בדרך כלל מוגדרת בחוק/תקנות, ונשארת KEEP ללא תלות בטכנולוגיה. (2) סיור פנימי שוטף של צוות האחזקה (יומי/שבועי) — לרוב אין לו תקן חיצוני שמגדיר תדירות/פרוטוקול מדויק, והוא הצטבר כנוהל/Best Practice. שכבה (2) היא המועמדת הטבעית לצמצום, אך מהסיבה הטכנית שבסעיף הזה (פער כיסוי חיישנים) — לא מהיעדר חובה רגולטורית.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>5. הסבר עמודות מפת ההחלטות</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>מערכת / ציוד / משימה</t>
         </is>
       </c>
-      <c r="B19" s="30" t="inlineStr">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>כפי שמופיעים בתוכנית האחזקה המקורית (12 לשוניות, 230 משימות) — שומר על שקיפות מלאה מול המקור.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="29" t="inlineStr">
-        <is>
-          <t>תדירות נוכחית / מופעים לשנה (היום)</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>התדירות כפי שנקבעה היום בתוכנית האחזקה, מתורגמת למספר מופעים שנתי.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="29" t="inlineStr">
-        <is>
-          <t>מה נבדק בפועל</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>תמצית הצ'ק-ליסט המקורי לאותה משימה.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="29" t="inlineStr">
-        <is>
-          <t>מקור החובה (Compliance)</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>הסיבה שבגללה המשימה קיימת: תקן ישראלי, חוק, הוראות יצרן, דרישת ביטוח, SLA או נוהל פנימי. זהו הבסיס לכל החלטת KEEP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>נתון קיים בבקר/BMS?</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>האם המידע הדרוש להערכת מצב המערכת כבר מגיע היום מבקר/רכזת/תוכנת ניהול קיימת.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="29" t="inlineStr">
-        <is>
-          <t>חיישן IoT נדרש</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>אם המידע חסר — איזה חיישן זול נדרש כדי להשלים אותו (רטט, דליפה, מילוי, הפרש לחץ וכו').</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t>בדיקה פיזית חובה עפ"י דין/תקן?</t>
+          <t>תדירות נוכחית / מופעים לשנה (היום)</t>
         </is>
       </c>
       <c r="B25" s="30" t="inlineStr">
         <is>
-          <t>דגל Compliance מפורש — אם כן, לא מוצעת החלטת SKIP למשימה, ללא תלות ביכולת הטכנולוגית.</t>
+          <t>התדירות כפי שנקבעה היום בתוכנית האחזקה, מתורגמת למספר מופעים שנתי.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="29" t="inlineStr">
         <is>
-          <t>ניתן למעבר לניהול מבוסס חריגות?</t>
+          <t>מה נבדק בפועל</t>
         </is>
       </c>
       <c r="B26" s="30" t="inlineStr">
         <is>
-          <t>הערכה כללית (כן/חלקי/לא) של מידת ההתאמה של המשימה למודל Condition-Based.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
+          <t>תמצית הצ'ק-ליסט המקורי לאותה משימה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>החלטת ברירת מחדל</t>
+          <t>מקור החובה (Compliance)</t>
         </is>
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>אחת מארבע ההחלטות (KEEP/SKIP/INSPECT/ACT), עם צביעה תואמת.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
+          <t>הסיבה שבגללה המשימה קיימת: תקן ישראלי, חוק, הוראות יצרן, דרישת ביטוח, SLA או נוהל פנימי. זהו הבסיס לכל החלטת KEEP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>תנאי SKIP / INSPECT / ACT</t>
+          <t>נתון קיים בבקר/BMS?</t>
         </is>
       </c>
       <c r="B28" s="30" t="inlineStr">
         <is>
-          <t>הלוגיקה בפועל: מתי המנוע מדלג, מתי הוא שולח לבדיקה מופחתת, ומתי הוא פותח קריאת שירות/פעולה.</t>
+          <t>האם המידע הדרוש להערכת מצב המערכת כבר מגיע היום מבקר/רכזת/תוכנת ניהול קיימת.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="29" t="inlineStr">
         <is>
-          <t>זמן ביצוע (דק') / מופעים חזויים / שעות בשנה</t>
+          <t>חיישן IoT נדרש</t>
         </is>
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>הערכות MVP לחישוב חיסכון פוטנציאלי — ראו הנחות עבודה בסעיף 5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="28" t="inlineStr">
-        <is>
-          <t>5. הנחות עבודה ומגבלות (MVP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="45" customHeight="1">
+          <t>אם המידע חסר — איזה חיישן זול נדרש כדי להשלים אותו (רטט, דליפה, מילוי, הפרש לחץ וכו').</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>בדיקה פיזית חובה עפ"י דין/תקן?</t>
+        </is>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>דגל Compliance מפורש — אם כן, לא מוצעת החלטת SKIP למשימה, ללא תלות ביכולת הטכנולוגית.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>ניתן למעבר לניהול מבוסס חריגות?</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="inlineStr">
+        <is>
+          <t>הערכה כללית (כן/חלקי/לא) של מידת ההתאמה של המשימה למודל Condition-Based.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
       <c r="A32" s="29" t="inlineStr">
         <is>
-          <t>•</t>
+          <t>החלטת ברירת מחדל</t>
         </is>
       </c>
       <c r="B32" s="30" t="inlineStr">
         <is>
-          <t>אומדני 'זמן ביצוע' ו'מופעים חזויים' הם הערכות סבירות של צוות הפיתוח בשלב Blueprint, ולא נתוני אמת נמדדים — מטרתן לבנות מודל חישוב שניתן להזין אליו בהמשך נתוני זמן אמיתיים (למשל ממגדלי הארבעה).</t>
+          <t>אחת מארבע ההחלטות (KEEP/SKIP/INSPECT/ACT), עם צביעה תואמת.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="29" t="inlineStr">
         <is>
+          <t>תנאי SKIP / INSPECT / ACT</t>
+        </is>
+      </c>
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>הלוגיקה בפועל: מתי המנוע מדלג, מתי הוא שולח לבדיקה מופחתת, ומתי הוא פותח קריאת שירות/פעולה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>זמן ביצוע (דק') / מופעים חזויים / שעות בשנה</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>הערכות MVP לחישוב חיסכון פוטנציאלי — ראו הנחות עבודה בסעיף 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>6. הנחות עבודה ומגבלות (MVP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B33" s="30" t="inlineStr">
+      <c r="B37" s="30" t="inlineStr">
+        <is>
+          <t>אומדני 'זמן ביצוע' ו'מופעים חזויים' הם הערכות סבירות של צוות הפיתוח בשלב Blueprint, ולא נתוני אמת נמדדים — מטרתן לבנות מודל חישוב שניתן להזין אליו בהמשך נתוני זמן אמיתיים (למשל ממגדלי הארבעה).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
         <is>
           <t>כל שורת KEEP מייצגת בכוונה חיסכון אפס או נמוך — זו דוגמה מכוונת לכך שהמנוע אינו ממליץ לבטל משימה רק כי קיימת טכנולוגיה, כאשר מקור החובה חיצוני ומחייב.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="29" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="29" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B34" s="30" t="inlineStr">
+      <c r="B39" s="30" t="inlineStr">
         <is>
           <t>שורות 'סיור ביטחון' מסומנות באזהרה מפורשת: כל צמצום מותנה באישור מראש של גורם הביטחון/הביטוח של הבניין — לא רק ביכולת הטכנולוגית, בהתאם לעיקרון הזהירות שהוגדר במסמך החזון.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="29" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="inlineStr">
-        <is>
-          <t>המשימות שנבחרו (36 מתוך 230) הן אלה בעלות פוטנציאל ההשפעה הגבוה ביותר (תדירות גבוהה + פוטנציאל אוטומציה) — הרחבה ליתר המשימות היא שלב 2 של התהליך.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="29" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B36" s="30" t="inlineStr">
-        <is>
-          <t>מקור החובה (Compliance) מבוסס על ידע כללי בתחום התקינה בישראל (ת"י 1220 ודומיו) ואינו מהווה ייעוץ משפטי/הנדסי — יש לאמת מול יועץ בטיחות/חשמל/כיבוי אש מוסמך לפני יישום בפועל.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="28" t="inlineStr">
-        <is>
-          <t>6. השלבים הבאים (מתוך מסמך החזון)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="29" t="inlineStr">
-        <is>
-          <t>→</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="inlineStr">
-        <is>
-          <t>הרחבת המטריצה ליתר 194 המשימות בתוכנית האחזקה (ולתוכנית הניקיון, כשתתקבל).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="29" t="inlineStr">
         <is>
-          <t>→</t>
+          <t>•</t>
         </is>
       </c>
       <c r="B40" s="30" t="inlineStr">
         <is>
-          <t>אימות מול נתוני אמת ממגדלי הארבעה — זמני ביצוע בפועל, מפת חיישנים/בקרים קיימת בפועל בכל מגדל.</t>
+          <t>המשימות שנבחרו (36 מתוך 230) הן אלה בעלות פוטנציאל ההשפעה הגבוה ביותר (תדירות גבוהה + פוטנציאל אוטומציה) — הרחבה ליתר המשימות היא שלב 2 של התהליך.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="29" t="inlineStr">
         <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>מקור החובה (Compliance) מבוסס על ידע כללי בתחום התקינה בישראל (ת"י 1220 ודומיו) ואינו מהווה ייעוץ משפטי/הנדסי — יש לאמת מול יועץ בטיחות/חשמל/כיבוי אש מוסמך לפני יישום בפועל.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
+          <t>7. השלבים הבאים (מתוך מסמך החזון + ממצאי הסיור במגדלי הארבעה)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
           <t>→</t>
         </is>
       </c>
-      <c r="B41" s="30" t="inlineStr">
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>הרחבת המטריצה ליתר 194 המשימות בתוכנית האחזקה (ולתוכנית הניקיון, כשתתקבל).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="29" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>אימות מול נתוני אמת ממגדלי הארבעה — זמני ביצוע בפועל, מפת חיישנים/בקרים קיימת בפועל בכל מגדל.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="B46" s="30" t="inlineStr">
+        <is>
+          <t>בירור טכני מול G1 הוטלו (מתחזקי מערכת הבקרה, פלטפורמת Trend/IQ-4): קיום ממשק BACnet/OPC או גישת קריאה למסד הנתונים/Trend log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="29" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="B47" s="30" t="inlineStr">
+        <is>
+          <t>בירור מול Visitt לגבי גישת API/ייצוא להיסטוריית המשימות שכבר קיימת בפועל בבניין — מקור נתוני אמת מהימן לכיול המודל.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="29" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="B48" s="30" t="inlineStr">
+        <is>
+          <t>מיפוי פערי כיסוי חיישנים לכל שורת INSPECT (עיקרון סעיף 4) — לא רק "יש בקר" אלא "אילו כשלים ספציפיים הבקר הקיים באמת מזהה".</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="29" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="B49" s="30" t="inlineStr">
         <is>
           <t>בניית Decision Engine V1 היברידי: שכבת Rules (Compliance) + שכבת Analytics/ML (זיהוי חריגות) + שכבת Generative AI (הסברים והמלצות).</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="29" t="inlineStr">
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="29" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="B42" s="30" t="inlineStr">
+      <c r="B50" s="30" t="inlineStr">
         <is>
           <t>בניית מסך Dashboard יומי ('BUILDING OPERATIONS — TODAY') המציג KEEP/SKIP/INSPECT/ACT לכל בניין בזמן אמת.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A38:B38"/>
+  <mergeCells count="8">
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A36:B36"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A31:B31"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A12:B12"/>

</xml_diff>